<commit_message>
corrected host scientific name
</commit_message>
<xml_diff>
--- a/example_files/zika_virus_test_metadata.xlsx
+++ b/example_files/zika_virus_test_metadata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skasambula\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skasambula\example_data\example_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9F4D20C-550F-4C83-B2A1-DE91B2BE7AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1098F20-2B54-4114-BECC-AA6B224D7281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BC45BC39-EA9A-48B3-A412-1DBB9FBA7354}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="111">
   <si>
     <t>id</t>
   </si>
@@ -306,9 +306,6 @@
     <t>Kenya</t>
   </si>
   <si>
-    <t>Homosapiens</t>
-  </si>
-  <si>
     <t>test_zika_006</t>
   </si>
   <si>
@@ -364,6 +361,12 @@
   </si>
   <si>
     <t>CNR Arbovirus, CNR Arbovirus</t>
+  </si>
+  <si>
+    <t>Homo sapiens</t>
+  </si>
+  <si>
+    <t>Aedes aegypti</t>
   </si>
 </sst>
 </file>
@@ -729,8 +732,8 @@
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
     <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.5546875" customWidth="1"/>
-    <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="72.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.77734375" customWidth="1"/>
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -993,13 +996,13 @@
         <v>46235</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:82" x14ac:dyDescent="0.3">
@@ -1013,13 +1016,13 @@
         <v>46236</v>
       </c>
       <c r="D3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:82" x14ac:dyDescent="0.3">
@@ -1036,10 +1039,10 @@
         <v>88</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:82" x14ac:dyDescent="0.3">
@@ -1056,10 +1059,10 @@
         <v>88</v>
       </c>
       <c r="E5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:82" x14ac:dyDescent="0.3">
@@ -1076,15 +1079,15 @@
         <v>88</v>
       </c>
       <c r="E6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F6" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
         <v>87</v>
@@ -1093,18 +1096,18 @@
         <v>46236</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
         <v>87</v>
@@ -1113,73 +1116,73 @@
         <v>46236</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" s="1">
         <v>46235</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C10" s="1">
         <v>46235</v>
       </c>
       <c r="D10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" t="s">
         <v>109</v>
-      </c>
-      <c r="F10" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" t="s">
         <v>95</v>
-      </c>
-      <c r="B11" t="s">
-        <v>96</v>
       </c>
       <c r="C11" s="1">
         <v>46235</v>
       </c>
       <c r="D11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" t="s">
         <v>109</v>
-      </c>
-      <c r="F11" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>